<commit_message>
Show exit net debt in returns bridge and sensitivity, use synthetic wording, add limitations and downside AI note
</commit_message>
<xml_diff>
--- a/model/PE_Value_Creation_Model_synthetic.xlsx
+++ b/model/PE_Value_Creation_Model_synthetic.xlsx
@@ -20538,7 +20538,7 @@
     <t xml:space="preserve">Synthetic historical results and entry baseline</t>
   </si>
   <si>
-    <t xml:space="preserve">Illustrative historical data only. The fictional company did not report these figures. USD millions.</t>
+    <t xml:space="preserve">Illustrative historical data only. The synthetic company did not report these figures. USD millions.</t>
   </si>
   <si>
     <t xml:space="preserve">EBITDA margin</t>
@@ -20850,7 +20850,7 @@
     <t xml:space="preserve">Exit fees ($m)</t>
   </si>
   <si>
-    <t xml:space="preserve">Exit gross debt ($m)</t>
+    <t xml:space="preserve">Exit net debt: gross debt less cash ($m)</t>
   </si>
   <si>
     <t xml:space="preserve">Exit equity proceeds ($m)</t>
@@ -21087,7 +21087,7 @@
     <t xml:space="preserve">Exit sponsor proceeds bridge</t>
   </si>
   <si>
-    <t xml:space="preserve">Exit EV less fee and debt plus retained cash equals exit equity proceeds.</t>
+    <t xml:space="preserve">Exit EV less exit fees and net debt (gross debt less cash) equals exit equity proceeds.</t>
   </si>
   <si>
     <t xml:space="preserve">Dashboard enterprise value bridge</t>
@@ -21324,7 +21324,7 @@
     <t xml:space="preserve">FY2025 revenue and EBITDA</t>
   </si>
   <si>
-    <t xml:space="preserve">Illustrative scale for a fictional mid-market services case.</t>
+    <t xml:space="preserve">Illustrative scale for a synthetic mid-market services case.</t>
   </si>
   <si>
     <t xml:space="preserve">Operating scenarios</t>
@@ -22287,11 +22287,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="4707499"/>
-        <c:axId val="37530018"/>
+        <c:axId val="42849437"/>
+        <c:axId val="23834942"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="4707499"/>
+        <c:axId val="42849437"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -22357,7 +22357,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37530018"/>
+        <c:crossAx val="23834942"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -22365,7 +22365,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="37530018"/>
+        <c:axId val="23834942"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -22441,7 +22441,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4707499"/>
+        <c:crossAx val="42849437"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -26543,7 +26543,7 @@
         <v>290</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">Returns!D20-Returns!D21-Returns!D22+'Cash Flow &amp; Debt'!H23-Returns!D23</f>
+        <f aca="false">Returns!D20-Returns!D21-Returns!D22-Returns!D23</f>
         <v>0</v>
       </c>
       <c r="E9" s="46" t="str">
@@ -30358,16 +30358,16 @@
         <v>212</v>
       </c>
       <c r="D22" s="16" t="n">
-        <f aca="false">'Cash Flow &amp; Debt'!H22</f>
-        <v>17.9706982621574</v>
+        <f aca="false">'Cash Flow &amp; Debt'!H24</f>
+        <v>15.2163169882128</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C23" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="D23" s="19" t="n">
-        <f aca="false">D20-D21-D22+'Cash Flow &amp; Debt'!H23</f>
+      <c r="D23" s="20" t="n">
+        <f aca="false">D20-D21-D22</f>
         <v>210.0941281434</v>
       </c>
     </row>
@@ -30561,23 +30561,23 @@
         <v>19.3448361981688</v>
       </c>
       <c r="D10" s="23" t="n">
-        <f aca="false">(($C10*D$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C10*D$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>1.58980167858622</v>
       </c>
       <c r="E10" s="23" t="n">
-        <f aca="false">(($C10*E$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C10*E$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>1.81043978729805</v>
       </c>
       <c r="F10" s="23" t="n">
-        <f aca="false">(($C10*F$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C10*F$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.03107789600988</v>
       </c>
       <c r="G10" s="23" t="n">
-        <f aca="false">(($C10*G$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C10*G$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.25171600472171</v>
       </c>
       <c r="H10" s="23" t="n">
-        <f aca="false">(($C10*H$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C10*H$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.47235411343355</v>
       </c>
       <c r="J10" s="26" t="n">
@@ -30590,23 +30590,23 @@
         <v>21.0517335097719</v>
       </c>
       <c r="D11" s="23" t="n">
-        <f aca="false">(($C11*D$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C11*D$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>1.74554622591222</v>
       </c>
       <c r="E11" s="23" t="n">
-        <f aca="false">(($C11*E$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C11*E$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>1.9856524030398</v>
       </c>
       <c r="F11" s="23" t="n">
-        <f aca="false">(($C11*F$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C11*F$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.22575858016738</v>
       </c>
       <c r="G11" s="23" t="n">
-        <f aca="false">(($C11*G$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C11*G$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.46586475729496</v>
       </c>
       <c r="H11" s="23" t="n">
-        <f aca="false">(($C11*H$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C11*H$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.70597093442255</v>
       </c>
       <c r="J11" s="26" t="n">
@@ -30619,23 +30619,23 @@
         <v>22.758630821375</v>
       </c>
       <c r="D12" s="23" t="n">
-        <f aca="false">(($C12*D$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C12*D$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>1.90129077323822</v>
       </c>
       <c r="E12" s="23" t="n">
-        <f aca="false">(($C12*E$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C12*E$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.16086501878155</v>
       </c>
       <c r="F12" s="23" t="n">
-        <f aca="false">(($C12*F$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C12*F$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.42043926432488</v>
       </c>
       <c r="G12" s="23" t="n">
-        <f aca="false">(($C12*G$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C12*G$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.68001350986821</v>
       </c>
       <c r="H12" s="23" t="n">
-        <f aca="false">(($C12*H$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C12*H$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.93958775541155</v>
       </c>
       <c r="J12" s="26" t="n">
@@ -30648,23 +30648,23 @@
         <v>24.4655281329781</v>
       </c>
       <c r="D13" s="23" t="n">
-        <f aca="false">(($C13*D$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C13*D$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.05703532056422</v>
       </c>
       <c r="E13" s="23" t="n">
-        <f aca="false">(($C13*E$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C13*E$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.3360776345233</v>
       </c>
       <c r="F13" s="23" t="n">
-        <f aca="false">(($C13*F$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C13*F$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.61511994848238</v>
       </c>
       <c r="G13" s="23" t="n">
-        <f aca="false">(($C13*G$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C13*G$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.89416226244146</v>
       </c>
       <c r="H13" s="23" t="n">
-        <f aca="false">(($C13*H$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C13*H$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>3.17320457640054</v>
       </c>
       <c r="J13" s="26" t="n">
@@ -30677,23 +30677,23 @@
         <v>26.1724254445812</v>
       </c>
       <c r="D14" s="23" t="n">
-        <f aca="false">(($C14*D$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C14*D$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.21277986789021</v>
       </c>
       <c r="E14" s="23" t="n">
-        <f aca="false">(($C14*E$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C14*E$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.51129025026505</v>
       </c>
       <c r="F14" s="23" t="n">
-        <f aca="false">(($C14*F$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C14*F$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>2.80980063263988</v>
       </c>
       <c r="G14" s="23" t="n">
-        <f aca="false">(($C14*G$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C14*G$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>3.10831101501471</v>
       </c>
       <c r="H14" s="23" t="n">
-        <f aca="false">(($C14*H$9)*(1-Controls!$D$24)-Returns!$D$22+'Cash Flow &amp; Debt'!$H$23)/Returns!$D$16</f>
+        <f aca="false">(($C14*H$9)*(1-Controls!$D$24)-Returns!$D$22)/Returns!$D$16</f>
         <v>3.40682139738954</v>
       </c>
       <c r="J14" s="26" t="n">

</xml_diff>